<commit_message>
Refactor documentation assets and update README for clarity and organization
</commit_message>
<xml_diff>
--- a/BandColorConvention/BandColorConvention.xlsx
+++ b/BandColorConvention/BandColorConvention.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\TechnicalDocumentation\BandColorConvention\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF79B81-C232-4A45-B393-6822E6D17B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5321A23F-4669-4B11-B1A5-9035BC78ABD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
+    <workbookView xWindow="570" yWindow="645" windowWidth="28230" windowHeight="14835" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Document Style" sheetId="4" r:id="rId1"/>
@@ -80,9 +80,6 @@
     <t>Keys, Guitar, Vocals</t>
   </si>
   <si>
-    <t>Bass, Vocals</t>
-  </si>
-  <si>
     <t>Position</t>
   </si>
   <si>
@@ -138,6 +135,9 @@
   </si>
   <si>
     <t>Vocals</t>
+  </si>
+  <si>
+    <t>Bass</t>
   </si>
 </sst>
 </file>
@@ -599,10 +599,10 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>6</v>
@@ -616,10 +616,10 @@
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>11</v>
@@ -630,30 +630,30 @@
         <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>25</v>
-      </c>
       <c r="E3" s="3" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A4" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>27</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>28</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>12</v>
@@ -667,13 +667,13 @@
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>30</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="33.75" x14ac:dyDescent="0.5">
@@ -684,10 +684,10 @@
         <v>2</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>12</v>
@@ -695,16 +695,16 @@
     </row>
     <row r="7" spans="1:5" ht="33.75" x14ac:dyDescent="0.5">
       <c r="A7" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>13</v>

</xml_diff>